<commit_message>
Applied new estimates and new initPop -the update included update of the do files for alignment targets, which is now also have improved format and produce ts plots in DoFilesTargets/TargetsPlots -updated documentation
</commit_message>
<xml_diff>
--- a/input/PL/reg_RMSE.xlsx
+++ b/input/PL/reg_RMSE.xlsx
@@ -6,7 +6,7 @@
     <workbookView activeTab="0"/>
   </bookViews>
   <sheets>
-    <sheet name="PL" sheetId="1" r:id="rId2"/>
+    <sheet name="RMSE" sheetId="1" r:id="rId2"/>
   </sheets>
   <calcPr calcId="125725" fullCalcOnLoad="true"/>
 </workbook>
@@ -16,9 +16,6 @@
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="7" uniqueCount="7">
   <si>
     <t>REGRESSOR</t>
-  </si>
-  <si>
-    <t>COEFFICIENT</t>
   </si>
   <si>
     <t>W1fa</t>
@@ -34,6 +31,9 @@
   </si>
   <si>
     <t>I3</t>
+  </si>
+  <si>
+    <t>COEFFICIENT</t>
   </si>
 </sst>
 </file>
@@ -54,7 +54,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -62,12 +62,14 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border/>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="true"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -77,7 +79,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:B7"/>
+  <dimension ref="A1:B6"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -85,46 +87,46 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>1</v>
+        <v>6</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
-      <c r="B2">
+      <c r="B2" s="1">
         <v>0.70939942835081815</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
-      <c r="B3">
+      <c r="B3" s="1">
         <v>0.74855881605590946</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
-      <c r="B4">
+      <c r="B4" s="1">
         <v>0.74855881605590946</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
-      <c r="B5">
+      <c r="B5" s="1">
         <v>0.74855881605590946</v>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" t="s">
-        <v>6</v>
+    <row r="6">
+      <c r="A6" t="s">
+        <v>5</v>
       </c>
-      <c r="B7">
+      <c r="B6" s="1">
         <v>0.72647449677507081</v>
       </c>
     </row>

</xml_diff>